<commit_message>
Sync educacion_tasas, piramide, cobertura y glosarios
</commit_message>
<xml_diff>
--- a/output/graficos_educacion_tasas/comunal_e_mat_a_2018_antofagasta.xlsx
+++ b/output/graficos_educacion_tasas/comunal_e_mat_a_2018_antofagasta.xlsx
@@ -1,46 +1,137 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="comunas" sheetId="1" r:id="rId1"/>
+    <sheet name="Comunas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comunas'!$A$1:$B$10</definedName>
+  </definedNames>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t xml:space="preserve">Comuna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antofagasta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">María Elena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mejillones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ollagüe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Pedro de Atacama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sierra Gorda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taltal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tocopilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de creación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-27 19:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIT - MDSF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagen asociada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comunal_e_mat_a_2018_antofagasta.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa de matrícula población de 0 a 24 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidad territorial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antofagasta (Comunal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
       <b/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00135A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,21 +139,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -112,10 +219,6 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -141,15 +244,12 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -175,6 +275,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -350,113 +451,168 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="22.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Comuna</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Antofagasta</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>69.09551999999999</v>
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>69.1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Calama</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>67.55905</v>
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>67.56</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>María Elena</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>67.20344</v>
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>67.2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Mejillones</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>64.65125999999999</v>
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>64.65</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ollagüe</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>72.85714</v>
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>72.86</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>San Pedro de Atacama</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>66.85202</v>
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>66.85</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sierra Gorda</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>66.66667</v>
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>66.67</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Taltal</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>73.22141000000001</v>
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>73.22</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Tocopilla</t>
-        </is>
-      </c>
-      <c r="B10">
-        <v>69.47235000000001</v>
+      <c r="A10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>69.47</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B10"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="24.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="60.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>